<commit_message>
Suppression des fichiers temporaires excel
</commit_message>
<xml_diff>
--- a/imports/Classe.xlsx
+++ b/imports/Classe.xlsx
@@ -701,7 +701,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="13.5" hidden="1" customHeight="1">
+    <row r="2" ht="13.5" customHeight="1">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -730,7 +730,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="13.5" hidden="1" customHeight="1">
+    <row r="3" ht="13.5" customHeight="1">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -759,7 +759,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" ht="13.5" hidden="1" customHeight="1">
+    <row r="4" ht="13.5" customHeight="1">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" ht="13.5" hidden="1" customHeight="1">
+    <row r="5" ht="13.5" customHeight="1">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -817,7 +817,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" ht="13.5" hidden="1" customHeight="1">
+    <row r="6" ht="13.5" customHeight="1">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -875,7 +875,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" ht="13.5" hidden="1" customHeight="1">
+    <row r="8" ht="13.5" customHeight="1">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -904,7 +904,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" ht="13.5" hidden="1" customHeight="1">
+    <row r="9" ht="13.5" customHeight="1">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -933,7 +933,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" ht="13.5" hidden="1" customHeight="1">
+    <row r="10" ht="13.5" customHeight="1">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -962,7 +962,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" ht="13.5" hidden="1" customHeight="1">
+    <row r="11" ht="13.5" customHeight="1">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -991,7 +991,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" ht="13.5" hidden="1" customHeight="1">
+    <row r="12" ht="13.5" customHeight="1">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1020,7 +1020,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" ht="13.5" hidden="1" customHeight="1">
+    <row r="13" ht="13.5" customHeight="1">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" ht="13.5" hidden="1" customHeight="1">
+    <row r="14" ht="13.5" customHeight="1">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" ht="13.5" hidden="1" customHeight="1">
+    <row r="15" ht="13.5" customHeight="1">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1108,13 +1108,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I15">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="PRIMC9"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I15"/>
   <sortState ref="A1:H15" columnSort="0">
     <sortCondition sortBy="value" descending="0" ref="A1:A15"/>
   </sortState>

</xml_diff>